<commit_message>
add MK I behemoth data (levels + skills) and fix material mappings
</commit_message>
<xml_diff>
--- a/src/data/excel/behemoth_levels.xlsx
+++ b/src/data/excel/behemoth_levels.xlsx
@@ -7,8 +7,6 @@
     <sheet name="MK III" sheetId="2" r:id="rId2"/>
     <sheet name="MK IV" sheetId="3" r:id="rId3"/>
     <sheet name="MK I" sheetId="4" r:id="rId4"/>
-    <sheet name="MK II" sheetId="5" r:id="rId5"/>
-    <sheet name="MK V" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -10495,7 +10493,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F201"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10525,16 +10523,16 @@
         <v>MK I</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D2" t="str">
-        <v>Placeholder</v>
+        <v>+192, +115, +1,152</v>
       </c>
       <c r="E2">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -10545,163 +10543,3981 @@
         <v>MK I</v>
       </c>
       <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="str">
+        <v>+248, +149, +1,488</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="str">
+        <v>+300, +180, +1,800</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="str">
+        <v>+356, +214, +2,136</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
+        <v>+408, +245, +2,450</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="str">
+        <v>+464, +278, +2,780</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="str">
+        <v>+516, +310, +3,100</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="str">
+        <v>+572, +343, +3,430</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="str">
+        <v>+624, +374, +3,740</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="str">
+        <v>+680, +408, +4,080</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="str">
+        <v>+732, +439, +4,390</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="str">
+        <v>+788, +473, +4,730</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="str">
+        <v>+840, +504, +5,040</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="str">
+        <v>+892, +535, +5,350</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16" t="str">
+        <v>+948, +569, +5,690</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17" t="str">
+        <v>+1,000, +600, +6,000</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>+1,056, +634, +6,340</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>+1,108, +665, +6,650</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20" t="str">
+        <v>+1,164, +698, +6,980</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
         <v>20</v>
       </c>
-      <c r="D3" t="str">
-        <v>Placeholder</v>
-      </c>
-      <c r="E3">
-        <v>1.4</v>
-      </c>
-      <c r="F3">
-        <v>2000</v>
+      <c r="B21" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="str">
+        <v>+1,216, +730, +7,300</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C22">
+        <v>4</v>
+      </c>
+      <c r="D22" t="str">
+        <v>+1,248, +749, +7,490</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23" t="str">
+        <v>+1,312, +787, +7,870</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C24">
+        <v>4</v>
+      </c>
+      <c r="D24" t="str">
+        <v>+1,312, +787, +7,870</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25" t="str">
+        <v>+1,344, +806, +8,060</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26" t="str">
+        <v>+1,380, +828, +8,280</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27" t="str">
+        <v>+1,412, +847, +8,470</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28" t="str">
+        <v>+1,444, +866, +8,660</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C29">
+        <v>4</v>
+      </c>
+      <c r="D29" t="str">
+        <v>+1,476, +886, +8,860</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C30">
+        <v>4</v>
+      </c>
+      <c r="D30" t="str">
+        <v>+1,508, +905, +9,050</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31" t="str">
+        <v>+1,540, +924, +9,240</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+      <c r="D32" t="str">
+        <v>+1,572, +943, +9,430</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C33">
+        <v>4</v>
+      </c>
+      <c r="D33" t="str">
+        <v>+1,604, +962, +9,620</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34" t="str">
+        <v>+1,636, +982, +9,820</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35" t="str">
+        <v>+1,668, +1,001, +10,010</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36" t="str">
+        <v>+1,700, +1,020, +10,200</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="D37" t="str">
+        <v>+1,732, +1,039, +10,390</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>9100</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C38">
+        <v>4</v>
+      </c>
+      <c r="D38" t="str">
+        <v>+1,764, +1,058, +10,580</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C39">
+        <v>4</v>
+      </c>
+      <c r="D39" t="str">
+        <v>+1,800, +1,080, +10,800</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40" t="str">
+        <v>+1,832, +1,099, +10,990</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>9300</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="D41" t="str">
+        <v>+1,864, +1,118, +11,180</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>9300</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C42">
+        <v>4</v>
+      </c>
+      <c r="D42" t="str">
+        <v>+1,892, +1,135, +11,350</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C43">
+        <v>4</v>
+      </c>
+      <c r="D43" t="str">
+        <v>+1,920, +1,152, +11,520</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C44">
+        <v>4</v>
+      </c>
+      <c r="D44" t="str">
+        <v>+1,952, +1,171, +11,710</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45" t="str">
+        <v>+1,980, +1,188, +11,880</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>9700</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C46">
+        <v>4</v>
+      </c>
+      <c r="D46" t="str">
+        <v>+2,008, +1,205, +12,050</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>9800</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C47">
+        <v>4</v>
+      </c>
+      <c r="D47" t="str">
+        <v>+2,036, +1,222, +12,220</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>9800</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48" t="str">
+        <v>+2,064, +1,238, +12,380</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49" t="str">
+        <v>+2,096, +1,258, +12,580</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50" t="str">
+        <v>+2,124, +1,274, +12,740</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51" t="str">
+        <v>+2,152, +1,291, +12,910</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52" t="str">
+        <v>+2,180, +1,310, +13,100</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53" t="str">
+        <v>+2,210, +1,327, +13,270</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54" t="str">
+        <v>+2,240, +1,344, +13,440</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>10900</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55" t="str">
+        <v>+2,270, +1,361, +13,610</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>10900</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
+      </c>
+      <c r="D56" t="str">
+        <v>+2,300, +1,380, +13,800</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>11400</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C57">
+        <v>1</v>
+      </c>
+      <c r="D57" t="str">
+        <v>+2,330, +1,397, +13,970</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>11400</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58" t="str">
+        <v>+2,360, +1,414, +14,140</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C59">
+        <v>2</v>
+      </c>
+      <c r="D59" t="str">
+        <v>+2,380, +1,430, +14,300</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C60">
+        <v>3</v>
+      </c>
+      <c r="D60" t="str">
+        <v>+2,420, +1,450, +14,500</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C61">
+        <v>3</v>
+      </c>
+      <c r="D61" t="str">
+        <v>+2,400, +1,466, +14,660</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62" t="str">
+        <v>+2,460, +1,478, +14,780</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63" t="str">
+        <v>+2,480, +1,488, +14,880</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64" t="str">
+        <v>+2,500, +1,502, +15,020</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65" t="str">
+        <v>+2,520, +1,514, +15,140</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66" t="str">
+        <v>+2,540, +1,524, +15,240</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67" t="str">
+        <v>+2,560, +1,536, +15,360</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68" t="str">
+        <v>+2,580, +1,548, +15,480</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+      <c r="D69" t="str">
+        <v>+2,600, +1,560, +15,600</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+      <c r="D70" t="str">
+        <v>+2,620, +1,572, +15,720</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71" t="str">
+        <v>+2,660, +1,594, +15,940</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>15800</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+      <c r="D72" t="str">
+        <v>+2,660, +1,594, +15,940</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>15900</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+      <c r="D73" t="str">
+        <v>+2,680, +1,606, +16,060</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>15900</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74" t="str">
+        <v>+2,700, +1,630, +16,300</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>15900</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+      <c r="D75" t="str">
+        <v>+2,720, +1,630, +16,300</v>
+      </c>
+      <c r="E75">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>15900</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+      <c r="D76" t="str">
+        <v>+2,740, +1,642, +16,420</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C77">
+        <v>1</v>
+      </c>
+      <c r="D77" t="str">
+        <v>+2,750, +1,651, +16,510</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C78">
+        <v>1</v>
+      </c>
+      <c r="D78" t="str">
+        <v>+2,770, +1,663, +16,630</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>16100</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C79">
+        <v>1</v>
+      </c>
+      <c r="D79" t="str">
+        <v>+2,800, +1,678, +16,780</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>16100</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80" t="str">
+        <v>+2,810, +1,687, +16,870</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>16200</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81" t="str">
+        <v>+2,830, +1,699, +16,990</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>16200</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C82">
+        <v>1</v>
+      </c>
+      <c r="D82" t="str">
+        <v>+2,850, +1,709, +17,090</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C83">
+        <v>1</v>
+      </c>
+      <c r="D83" t="str">
+        <v>+2,870, +1,721, +17,210</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C84">
+        <v>1</v>
+      </c>
+      <c r="D84" t="str">
+        <v>+2,880, +1,730, +17,300</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>16900</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="D85" t="str">
+        <v>+2,900, +1,740, +17,400</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>16900</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C86">
+        <v>2</v>
+      </c>
+      <c r="D86" t="str">
+        <v>+2,920, +1,752, +17,520</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>17100</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C87">
+        <v>2</v>
+      </c>
+      <c r="D87" t="str">
+        <v>+2,940, +1,762, +17,620</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>17100</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C88">
+        <v>2</v>
+      </c>
+      <c r="D88" t="str">
+        <v>+2,960, +1,774, +17,740</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>17300</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C89">
+        <v>2</v>
+      </c>
+      <c r="D89" t="str">
+        <v>+2,970, +1,783, +17,830</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+      <c r="F89">
+        <v>17300</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C90">
+        <v>2</v>
+      </c>
+      <c r="D90" t="str">
+        <v>+2,990, +1,793, +17,930</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>17600</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C91">
+        <v>2</v>
+      </c>
+      <c r="D91" t="str">
+        <v>+3,010, +1,805, +18,050</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>17600</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C92">
+        <v>3</v>
+      </c>
+      <c r="D92" t="str">
+        <v>+3,020, +1,814, +18,140</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C93">
+        <v>3</v>
+      </c>
+      <c r="D93" t="str">
+        <v>+3,040, +1,824, +18,240</v>
+      </c>
+      <c r="E93">
+        <v>0</v>
+      </c>
+      <c r="F93">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C94">
+        <v>3</v>
+      </c>
+      <c r="D94" t="str">
+        <v>+3,060, +1,836, +18,360</v>
+      </c>
+      <c r="E94">
+        <v>0</v>
+      </c>
+      <c r="F94">
+        <v>18400</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C95">
+        <v>3</v>
+      </c>
+      <c r="D95" t="str">
+        <v>+3,080, +1,846, +18,460</v>
+      </c>
+      <c r="E95">
+        <v>0</v>
+      </c>
+      <c r="F95">
+        <v>18400</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C96">
+        <v>4</v>
+      </c>
+      <c r="D96" t="str">
+        <v>+3,100, +1,858, +18,580</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C97">
+        <v>4</v>
+      </c>
+      <c r="D97" t="str">
+        <v>+3,110, +1,867, +18,670</v>
+      </c>
+      <c r="E97">
+        <v>0</v>
+      </c>
+      <c r="F97">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C98">
+        <v>4</v>
+      </c>
+      <c r="D98" t="str">
+        <v>+3,130, +1,877, +18,770</v>
+      </c>
+      <c r="E98">
+        <v>0</v>
+      </c>
+      <c r="F98">
+        <v>19700</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C99">
+        <v>4</v>
+      </c>
+      <c r="D99" t="str">
+        <v>+3,150, +1,889, +18,890</v>
+      </c>
+      <c r="E99">
+        <v>0</v>
+      </c>
+      <c r="F99">
+        <v>19700</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+      <c r="D100" t="str">
+        <v>+3,160, +1,898, +18,980</v>
+      </c>
+      <c r="E100">
+        <v>0</v>
+      </c>
+      <c r="F100">
+        <v>20900</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+      <c r="D101" t="str">
+        <v>+3,180, +1,908, +19,080</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>20900</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C102">
+        <v>0</v>
+      </c>
+      <c r="D102" t="str">
+        <v>+3,190, +1,915, +19,150</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>25300</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C103">
+        <v>0</v>
+      </c>
+      <c r="D103" t="str">
+        <v>+3,200, +1,922, +19,220</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>25300</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C104">
+        <v>0</v>
+      </c>
+      <c r="D104" t="str">
+        <v>+3,220, +1,930, +19,300</v>
+      </c>
+      <c r="E104">
+        <v>0</v>
+      </c>
+      <c r="F104">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+      <c r="D105" t="str">
+        <v>+3,230, +1,937, +19,370</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C106">
+        <v>0</v>
+      </c>
+      <c r="D106" t="str">
+        <v>+3,240, +1,944, +19,400</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C107">
+        <v>0</v>
+      </c>
+      <c r="D107" t="str">
+        <v>+3,250, +1,951, +19,510</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C108">
+        <v>0</v>
+      </c>
+      <c r="D108" t="str">
+        <v>+3,260, +1,958, +19,580</v>
+      </c>
+      <c r="E108">
+        <v>0</v>
+      </c>
+      <c r="F108">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C109">
+        <v>0</v>
+      </c>
+      <c r="D109" t="str">
+        <v>+3,270, +1,963, +19,630</v>
+      </c>
+      <c r="E109">
+        <v>0</v>
+      </c>
+      <c r="F109">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C110">
+        <v>0</v>
+      </c>
+      <c r="D110" t="str">
+        <v>+3,280, +1,970, +19,700</v>
+      </c>
+      <c r="E110">
+        <v>0</v>
+      </c>
+      <c r="F110">
+        <v>25500</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C111">
+        <v>0</v>
+      </c>
+      <c r="D111" t="str">
+        <v>+3,300, +1,978, +19,780</v>
+      </c>
+      <c r="E111">
+        <v>0</v>
+      </c>
+      <c r="F111">
+        <v>25500</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C112">
+        <v>0</v>
+      </c>
+      <c r="D112" t="str">
+        <v>+3,310, +1,985, +19,850</v>
+      </c>
+      <c r="E112">
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>25500</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C113">
+        <v>0</v>
+      </c>
+      <c r="D113" t="str">
+        <v>+3,320, +1,920, +19,920</v>
+      </c>
+      <c r="E113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>25500</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C114">
+        <v>0</v>
+      </c>
+      <c r="D114" t="str">
+        <v>+3,330, +1,999, +19,990</v>
+      </c>
+      <c r="E114">
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>25600</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C115">
+        <v>0</v>
+      </c>
+      <c r="D115" t="str">
+        <v>+3,340, +2,006, +20,060</v>
+      </c>
+      <c r="E115">
+        <v>0</v>
+      </c>
+      <c r="F115">
+        <v>25600</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C116">
+        <v>0</v>
+      </c>
+      <c r="D116" t="str">
+        <v>+3,360, +2,014, +201140</v>
+      </c>
+      <c r="E116">
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>25700</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C117">
+        <v>0</v>
+      </c>
+      <c r="D117" t="str">
+        <v>+3,370, +2,021, +20,210</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>25700</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C118">
+        <v>0</v>
+      </c>
+      <c r="D118" t="str">
+        <v>+3,380, +2,028, +20,280</v>
+      </c>
+      <c r="E118">
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>25900</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C119">
+        <v>0</v>
+      </c>
+      <c r="D119" t="str">
+        <v>+3,390, +2,033, +20,330</v>
+      </c>
+      <c r="E119">
+        <v>0</v>
+      </c>
+      <c r="F119">
+        <v>25900</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C120">
+        <v>1</v>
+      </c>
+      <c r="D120" t="str">
+        <v>+3,400, +2,040, +20,400</v>
+      </c>
+      <c r="E120">
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C121">
+        <v>1</v>
+      </c>
+      <c r="D121" t="str">
+        <v>+3,412, +2,047, +20,470</v>
+      </c>
+      <c r="E121">
+        <v>0</v>
+      </c>
+      <c r="F121">
+        <v>26100</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C122">
+        <v>2</v>
+      </c>
+      <c r="D122" t="str">
+        <v>+3,424, +2,054, +20,540</v>
+      </c>
+      <c r="E122">
+        <v>0</v>
+      </c>
+      <c r="F122">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C123">
+        <v>2</v>
+      </c>
+      <c r="D123" t="str">
+        <v>+3,436, +2,062, +20,620</v>
+      </c>
+      <c r="E123">
+        <v>0</v>
+      </c>
+      <c r="F123">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C124">
+        <v>2</v>
+      </c>
+      <c r="D124" t="str">
+        <v>+3,444, +2,066, +20,660</v>
+      </c>
+      <c r="E124">
+        <v>0</v>
+      </c>
+      <c r="F124">
+        <v>27100</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C125">
+        <v>2</v>
+      </c>
+      <c r="D125" t="str">
+        <v>+3,456, +2,074, +20,740</v>
+      </c>
+      <c r="E125">
+        <v>0</v>
+      </c>
+      <c r="F125">
+        <v>27100</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C126">
+        <v>2</v>
+      </c>
+      <c r="D126" t="str">
+        <v>+3,464, +2,078, +20,780</v>
+      </c>
+      <c r="E126">
+        <v>0</v>
+      </c>
+      <c r="F126">
+        <v>27300</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C127">
+        <v>2</v>
+      </c>
+      <c r="D127" t="str">
+        <v>+3,476, +2,086, +20,860</v>
+      </c>
+      <c r="E127">
+        <v>0</v>
+      </c>
+      <c r="F127">
+        <v>27300</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C128">
+        <v>2</v>
+      </c>
+      <c r="D128" t="str">
+        <v>+3,484, +2,090, +20,900</v>
+      </c>
+      <c r="E128">
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>27600</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C129">
+        <v>2</v>
+      </c>
+      <c r="D129" t="str">
+        <v>+3,496, +2,098, +20,980</v>
+      </c>
+      <c r="E129">
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>27600</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C130">
+        <v>2</v>
+      </c>
+      <c r="D130" t="str">
+        <v>+3,508, +2,105, +21,050</v>
+      </c>
+      <c r="E130">
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>27900</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C131">
+        <v>2</v>
+      </c>
+      <c r="D131" t="str">
+        <v>+3,520, +2,112, +21,120</v>
+      </c>
+      <c r="E131">
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>27900</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C132">
+        <v>3</v>
+      </c>
+      <c r="D132" t="str">
+        <v>+3,528, +2,117, +21,170</v>
+      </c>
+      <c r="E132">
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>28300</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C133">
+        <v>3</v>
+      </c>
+      <c r="D133" t="str">
+        <v>+3,540, +2,124, +21,240</v>
+      </c>
+      <c r="E133">
+        <v>0</v>
+      </c>
+      <c r="F133">
+        <v>28300</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C134">
+        <v>3</v>
+      </c>
+      <c r="D134" t="str">
+        <v>+3,548, +2,129, +21,290</v>
+      </c>
+      <c r="E134">
+        <v>0</v>
+      </c>
+      <c r="F134">
+        <v>28800</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C135">
+        <v>3</v>
+      </c>
+      <c r="D135" t="str">
+        <v>+3,560, +2,136, +21,360</v>
+      </c>
+      <c r="E135">
+        <v>0</v>
+      </c>
+      <c r="F135">
+        <v>28800</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C136">
+        <v>4</v>
+      </c>
+      <c r="D136" t="str">
+        <v>+3,568, +2,141, +24,101</v>
+      </c>
+      <c r="E136">
+        <v>0</v>
+      </c>
+      <c r="F136">
+        <v>29500</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C137">
+        <v>4</v>
+      </c>
+      <c r="D137" t="str">
+        <v>+3,580, +2,148, +21,480</v>
+      </c>
+      <c r="E137">
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>29500</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C138">
+        <v>0</v>
+      </c>
+      <c r="D138" t="str">
+        <v>+3,592, +2,155, +21,550</v>
+      </c>
+      <c r="E138">
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>30400</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C139">
+        <v>0</v>
+      </c>
+      <c r="D139" t="str">
+        <v>+3,600, +2,160, +21,600</v>
+      </c>
+      <c r="E139">
+        <v>0</v>
+      </c>
+      <c r="F139">
+        <v>30400</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C140">
+        <v>1</v>
+      </c>
+      <c r="D140" t="str">
+        <v>+3,612, +2,167, +21,670</v>
+      </c>
+      <c r="E140">
+        <v>0</v>
+      </c>
+      <c r="F140">
+        <v>31900</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C141">
+        <v>1</v>
+      </c>
+      <c r="D141" t="str">
+        <v>+3,624, +2,174, +21,740</v>
+      </c>
+      <c r="E141">
+        <v>0</v>
+      </c>
+      <c r="F141">
+        <v>31900</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C142">
+        <v>3</v>
+      </c>
+      <c r="D142" t="str">
+        <v>+3,628, +2,177, +21,770</v>
+      </c>
+      <c r="E142">
+        <v>0</v>
+      </c>
+      <c r="F142">
+        <v>38700</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C143">
+        <v>3</v>
+      </c>
+      <c r="D143" t="str">
+        <v>+3,636, +2,182, +21,820</v>
+      </c>
+      <c r="E143">
+        <v>0</v>
+      </c>
+      <c r="F143">
+        <v>38700</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C144">
+        <v>3</v>
+      </c>
+      <c r="D144" t="str">
+        <v>+3,644, +2,186, +21,860</v>
+      </c>
+      <c r="E144">
+        <v>0</v>
+      </c>
+      <c r="F144">
+        <v>38800</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C145">
+        <v>3</v>
+      </c>
+      <c r="D145" t="str">
+        <v>+3,652, +2,191, +21,910</v>
+      </c>
+      <c r="E145">
+        <v>0</v>
+      </c>
+      <c r="F145">
+        <v>38800</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C146">
+        <v>3</v>
+      </c>
+      <c r="D146" t="str">
+        <v>+3,656, +2,194, +21,940</v>
+      </c>
+      <c r="E146">
+        <v>0</v>
+      </c>
+      <c r="F146">
+        <v>38900</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C147">
+        <v>3</v>
+      </c>
+      <c r="D147" t="str">
+        <v>+3,664, +2,198, +21,980</v>
+      </c>
+      <c r="E147">
+        <v>0</v>
+      </c>
+      <c r="F147">
+        <v>38900</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C148">
+        <v>4</v>
+      </c>
+      <c r="D148" t="str">
+        <v>+3,672, +2,203, +22,030</v>
+      </c>
+      <c r="E148">
+        <v>0</v>
+      </c>
+      <c r="F148">
+        <v>39100</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C149">
+        <v>4</v>
+      </c>
+      <c r="D149" t="str">
+        <v>+3,676, +2,206, +22,060</v>
+      </c>
+      <c r="E149">
+        <v>0</v>
+      </c>
+      <c r="F149">
+        <v>39100</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C150">
+        <v>4</v>
+      </c>
+      <c r="D150" t="str">
+        <v>+3,684, +2,210, +22,100</v>
+      </c>
+      <c r="E150">
+        <v>0</v>
+      </c>
+      <c r="F150">
+        <v>39300</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C151">
+        <v>4</v>
+      </c>
+      <c r="D151" t="str">
+        <v>+3,692, +2,215, +22,150</v>
+      </c>
+      <c r="E151">
+        <v>0</v>
+      </c>
+      <c r="F151">
+        <v>39300</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C152">
+        <v>4</v>
+      </c>
+      <c r="D152" t="str">
+        <v>+3,700, +2,220, +22,200</v>
+      </c>
+      <c r="E152">
+        <v>0</v>
+      </c>
+      <c r="F152">
+        <v>39600</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C153">
+        <v>4</v>
+      </c>
+      <c r="D153" t="str">
+        <v>+3,708, +2,225, +22,250</v>
+      </c>
+      <c r="E153">
+        <v>0</v>
+      </c>
+      <c r="F153">
+        <v>39600</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C154">
+        <v>0</v>
+      </c>
+      <c r="D154" t="str">
+        <v>+3,712, +2,227, +22,270</v>
+      </c>
+      <c r="E154">
+        <v>0</v>
+      </c>
+      <c r="F154">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C155">
+        <v>0</v>
+      </c>
+      <c r="D155" t="str">
+        <v>+3,720, +2,232, +22,320</v>
+      </c>
+      <c r="E155">
+        <v>0</v>
+      </c>
+      <c r="F155">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C156">
+        <v>0</v>
+      </c>
+      <c r="D156" t="str">
+        <v>+3,728, +2,237, +22,370</v>
+      </c>
+      <c r="E156">
+        <v>0</v>
+      </c>
+      <c r="F156">
+        <v>40600</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C157">
+        <v>0</v>
+      </c>
+      <c r="D157" t="str">
+        <v>+3,732, +2,239, +22,390</v>
+      </c>
+      <c r="E157">
+        <v>0</v>
+      </c>
+      <c r="F157">
+        <v>40600</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C158">
+        <v>1</v>
+      </c>
+      <c r="D158" t="str">
+        <v>+3,740, +2,244, +22,440</v>
+      </c>
+      <c r="E158">
+        <v>0</v>
+      </c>
+      <c r="F158">
+        <v>41400</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C159">
+        <v>1</v>
+      </c>
+      <c r="D159" t="str">
+        <v>+3,748, +2,249, +22,490</v>
+      </c>
+      <c r="E159">
+        <v>0</v>
+      </c>
+      <c r="F159">
+        <v>41400</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C160">
+        <v>2</v>
+      </c>
+      <c r="D160" t="str">
+        <v>+3,759, +2,254, +22,540</v>
+      </c>
+      <c r="E160">
+        <v>0</v>
+      </c>
+      <c r="F160">
+        <v>42600</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C161">
+        <v>2</v>
+      </c>
+      <c r="D161" t="str">
+        <v>+3,764, +2,258, +22,580</v>
+      </c>
+      <c r="E161">
+        <v>0</v>
+      </c>
+      <c r="F161">
+        <v>42600</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C162">
+        <v>3</v>
+      </c>
+      <c r="D162" t="str">
+        <v>+3,768, +2,261, +22,610</v>
+      </c>
+      <c r="E162">
+        <v>0</v>
+      </c>
+      <c r="F162">
+        <v>43900</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C163">
+        <v>3</v>
+      </c>
+      <c r="D163" t="str">
+        <v>+3,772, +2,263, +22,630</v>
+      </c>
+      <c r="E163">
+        <v>0</v>
+      </c>
+      <c r="F163">
+        <v>43900</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C164">
+        <v>4</v>
+      </c>
+      <c r="D164" t="str">
+        <v>+3,780, +2,268, +22,680</v>
+      </c>
+      <c r="E164">
+        <v>0</v>
+      </c>
+      <c r="F164">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C165">
+        <v>4</v>
+      </c>
+      <c r="D165" t="str">
+        <v>+3,788, +2,263, +22,630</v>
+      </c>
+      <c r="E165">
+        <v>0</v>
+      </c>
+      <c r="F165">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C166">
+        <v>4</v>
+      </c>
+      <c r="D166" t="str">
+        <v>+3,796, +2,278, +22,780</v>
+      </c>
+      <c r="E166">
+        <v>0</v>
+      </c>
+      <c r="F166">
+        <v>44200</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C167">
+        <v>4</v>
+      </c>
+      <c r="D167" t="str">
+        <v>+3,800, +2,280, +22,800</v>
+      </c>
+      <c r="E167">
+        <v>0</v>
+      </c>
+      <c r="F167">
+        <v>44200</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C168">
+        <v>4</v>
+      </c>
+      <c r="D168" t="str">
+        <v>+3,808, +2,285, +222,850</v>
+      </c>
+      <c r="E168">
+        <v>0</v>
+      </c>
+      <c r="F168">
+        <v>44300</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C169">
+        <v>4</v>
+      </c>
+      <c r="D169" t="str">
+        <v>+3,812, +2,287, +22,870</v>
+      </c>
+      <c r="E169">
+        <v>0</v>
+      </c>
+      <c r="F169">
+        <v>44300</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C170">
+        <v>4</v>
+      </c>
+      <c r="D170" t="str">
+        <v>+3,820, +2,292, +22,920</v>
+      </c>
+      <c r="E170">
+        <v>0</v>
+      </c>
+      <c r="F170">
+        <v>44600</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C171">
+        <v>4</v>
+      </c>
+      <c r="D171" t="str">
+        <v>+3,824, +2,294, +22,940</v>
+      </c>
+      <c r="E171">
+        <v>0</v>
+      </c>
+      <c r="F171">
+        <v>44600</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C172">
+        <v>0</v>
+      </c>
+      <c r="D172" t="str">
+        <v>+3,832, +2,299, +22,990</v>
+      </c>
+      <c r="E172">
+        <v>0</v>
+      </c>
+      <c r="F172">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C173">
+        <v>0</v>
+      </c>
+      <c r="D173" t="str">
+        <v>+3,840, +2,304, +23,040</v>
+      </c>
+      <c r="E173">
+        <v>0</v>
+      </c>
+      <c r="F173">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C174">
+        <v>0</v>
+      </c>
+      <c r="D174" t="str">
+        <v>+3,844, +2,306, +23,060</v>
+      </c>
+      <c r="E174">
+        <v>0</v>
+      </c>
+      <c r="F174">
+        <v>45400</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C175">
+        <v>0</v>
+      </c>
+      <c r="D175" t="str">
+        <v>+3,848, +2,309, +23,090</v>
+      </c>
+      <c r="E175">
+        <v>0</v>
+      </c>
+      <c r="F175">
+        <v>45400</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C176">
+        <v>1</v>
+      </c>
+      <c r="D176" t="str">
+        <v>+3,856, +2,314, +23,140</v>
+      </c>
+      <c r="E176">
+        <v>0</v>
+      </c>
+      <c r="F176">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C177">
+        <v>1</v>
+      </c>
+      <c r="D177" t="str">
+        <v>+3,864, +2,318, +23,180</v>
+      </c>
+      <c r="E177">
+        <v>0</v>
+      </c>
+      <c r="F177">
+        <v>46100</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C178">
+        <v>1</v>
+      </c>
+      <c r="D178" t="str">
+        <v>+3,868, +2,321, +23,210</v>
+      </c>
+      <c r="E178">
+        <v>0</v>
+      </c>
+      <c r="F178">
+        <v>46900</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C179">
+        <v>1</v>
+      </c>
+      <c r="D179" t="str">
+        <v>+3,876, +2,326, +23,260</v>
+      </c>
+      <c r="E179">
+        <v>0</v>
+      </c>
+      <c r="F179">
+        <v>46900</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C180">
+        <v>3</v>
+      </c>
+      <c r="D180" t="str">
+        <v>+3,880, +2,328, +23,280</v>
+      </c>
+      <c r="E180">
+        <v>0</v>
+      </c>
+      <c r="F180">
+        <v>48200</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C181">
+        <v>3</v>
+      </c>
+      <c r="D181" t="str">
+        <v>+3,888, +2,333, +23,330</v>
+      </c>
+      <c r="E181">
+        <v>0</v>
+      </c>
+      <c r="F181">
+        <v>48200</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C182">
+        <v>4</v>
+      </c>
+      <c r="D182" t="str">
+        <v>+3,892, +2,335, +23,350</v>
+      </c>
+      <c r="E182">
+        <v>0</v>
+      </c>
+      <c r="F182">
+        <v>54400</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C183">
+        <v>4</v>
+      </c>
+      <c r="D183" t="str">
+        <v>+3,896, +2,338, +23,380</v>
+      </c>
+      <c r="E183">
+        <v>0</v>
+      </c>
+      <c r="F183">
+        <v>59400</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C184">
+        <v>0</v>
+      </c>
+      <c r="D184" t="str">
+        <v>+3,904, +2,342, +23,420</v>
+      </c>
+      <c r="E184">
+        <v>0</v>
+      </c>
+      <c r="F184">
+        <v>65100</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C185">
+        <v>1</v>
+      </c>
+      <c r="D185" t="str">
+        <v>+3,912, +2,347, +23,470</v>
+      </c>
+      <c r="E185">
+        <v>0</v>
+      </c>
+      <c r="F185">
+        <v>71200</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C186">
+        <v>3</v>
+      </c>
+      <c r="D186" t="str">
+        <v>+3,916, +2,350, +23,500</v>
+      </c>
+      <c r="E186">
+        <v>0</v>
+      </c>
+      <c r="F186">
+        <v>78100</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C187">
+        <v>0</v>
+      </c>
+      <c r="D187" t="str">
+        <v>+3,920, +2,352, +23,520</v>
+      </c>
+      <c r="E187">
+        <v>0</v>
+      </c>
+      <c r="F187">
+        <v>85400</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C188">
+        <v>3</v>
+      </c>
+      <c r="D188" t="str">
+        <v>+3,928, +2,357, +23,570</v>
+      </c>
+      <c r="E188">
+        <v>0</v>
+      </c>
+      <c r="F188">
+        <v>93700</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C189">
+        <v>2</v>
+      </c>
+      <c r="D189" t="str">
+        <v>+3,932, +2,359, +23,590</v>
+      </c>
+      <c r="E189">
+        <v>0</v>
+      </c>
+      <c r="F189">
+        <v>102000</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C190">
+        <v>3</v>
+      </c>
+      <c r="D190" t="str">
+        <v>+3,940, +2,364, +23,640</v>
+      </c>
+      <c r="E190">
+        <v>0</v>
+      </c>
+      <c r="F190">
+        <v>113000</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C191">
+        <v>3</v>
+      </c>
+      <c r="D191" t="str">
+        <v>+3,944, +2,366, +23,660</v>
+      </c>
+      <c r="E191">
+        <v>0</v>
+      </c>
+      <c r="F191">
+        <v>123000</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C192">
+        <v>1</v>
+      </c>
+      <c r="D192" t="str">
+        <v>+3,948, +2,369, +23,690</v>
+      </c>
+      <c r="E192">
+        <v>0</v>
+      </c>
+      <c r="F192">
+        <v>136000</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C193">
+        <v>3</v>
+      </c>
+      <c r="D193" t="str">
+        <v>+3,956, +2,374, +23,740</v>
+      </c>
+      <c r="E193">
+        <v>0</v>
+      </c>
+      <c r="F193">
+        <v>148000</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C194">
+        <v>4</v>
+      </c>
+      <c r="D194" t="str">
+        <v>+3,960, +2,376, +23,760</v>
+      </c>
+      <c r="E194">
+        <v>0</v>
+      </c>
+      <c r="F194">
+        <v>164000</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C195">
+        <v>4</v>
+      </c>
+      <c r="D195" t="str">
+        <v>+3,968, +2,381, +23,810</v>
+      </c>
+      <c r="E195">
+        <v>0</v>
+      </c>
+      <c r="F195">
+        <v>179000</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C196">
+        <v>3</v>
+      </c>
+      <c r="D196" t="str">
+        <v>+3,972, +2,383, +23,830</v>
+      </c>
+      <c r="E196">
+        <v>0</v>
+      </c>
+      <c r="F196">
+        <v>198000</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C197">
+        <v>2</v>
+      </c>
+      <c r="D197" t="str">
+        <v>+3,980, +2,388, +23,880</v>
+      </c>
+      <c r="E197">
+        <v>0</v>
+      </c>
+      <c r="F197">
+        <v>217000</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C198">
+        <v>1</v>
+      </c>
+      <c r="D198" t="str">
+        <v>+3,984, +2,390, +23,900</v>
+      </c>
+      <c r="E198">
+        <v>0</v>
+      </c>
+      <c r="F198">
+        <v>241000</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C199">
+        <v>3</v>
+      </c>
+      <c r="D199" t="str">
+        <v>+3,988, +2,393, +23,930</v>
+      </c>
+      <c r="E199">
+        <v>0</v>
+      </c>
+      <c r="F199">
+        <v>263000</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C200">
+        <v>0</v>
+      </c>
+      <c r="D200" t="str">
+        <v>+3,996, +2,398, +23,398</v>
+      </c>
+      <c r="E200">
+        <v>0</v>
+      </c>
+      <c r="F200">
+        <v>295000</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="str">
+        <v>MK I</v>
+      </c>
+      <c r="C201">
+        <v>2</v>
+      </c>
+      <c r="D201" t="str">
+        <v>+4,000, +2,400, +24,000</v>
+      </c>
+      <c r="E201">
+        <v>0</v>
+      </c>
+      <c r="F201">
+        <v>322000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Level</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mk</v>
-      </c>
-      <c r="C1" t="str">
-        <v>PowerSerum</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Benefit</v>
-      </c>
-      <c r="E1" t="str">
-        <v>BenefitPct</v>
-      </c>
-      <c r="F1" t="str">
-        <v>PointsToUpgrade</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>MK II</v>
-      </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Placeholder</v>
-      </c>
-      <c r="E2">
-        <v>1.4</v>
-      </c>
-      <c r="F2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>MK II</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Placeholder</v>
-      </c>
-      <c r="E3">
-        <v>1.4</v>
-      </c>
-      <c r="F3">
-        <v>2000</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Level</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Mk</v>
-      </c>
-      <c r="C1" t="str">
-        <v>PowerSerum</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Benefit</v>
-      </c>
-      <c r="E1" t="str">
-        <v>BenefitPct</v>
-      </c>
-      <c r="F1" t="str">
-        <v>PointsToUpgrade</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>MK V</v>
-      </c>
-      <c r="C2">
-        <v>10</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Placeholder</v>
-      </c>
-      <c r="E2">
-        <v>1.4</v>
-      </c>
-      <c r="F2">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>MK V</v>
-      </c>
-      <c r="C3">
-        <v>20</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Placeholder</v>
-      </c>
-      <c r="E3">
-        <v>1.4</v>
-      </c>
-      <c r="F3">
-        <v>2000</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F201"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Behemoth MK V level costs (Serum) and always emit bonuses in converter
</commit_message>
<xml_diff>
--- a/src/data/excel/behemoth_levels.xlsx
+++ b/src/data/excel/behemoth_levels.xlsx
@@ -8,6 +8,7 @@
     <sheet name="MK IV" sheetId="3" r:id="rId3"/>
     <sheet name="MK II" sheetId="4" r:id="rId4"/>
     <sheet name="MK I" sheetId="5" r:id="rId5"/>
+    <sheet name="MK V" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -18552,4 +18553,4035 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F201"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F201"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Level</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Mk</v>
+      </c>
+      <c r="C1" t="str">
+        <v>PowerSerum</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Benefit</v>
+      </c>
+      <c r="E1" t="str">
+        <v>BenefitPct</v>
+      </c>
+      <c r="F1" t="str">
+        <v>PointsToUpgrade</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C45">
+        <v>1</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C47">
+        <v>1</v>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C54">
+        <v>2</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C55">
+        <v>2</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C56">
+        <v>2</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C57">
+        <v>2</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C58">
+        <v>2</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C59">
+        <v>2</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C60">
+        <v>2</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C61">
+        <v>2</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C62">
+        <v>3</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C63">
+        <v>3</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C65">
+        <v>3</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C66">
+        <v>3</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C68">
+        <v>3</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C69">
+        <v>3</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C71">
+        <v>3</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C72">
+        <v>3</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C73">
+        <v>3</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C74">
+        <v>3</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C75">
+        <v>3</v>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C76">
+        <v>3</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C77">
+        <v>3</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C78">
+        <v>3</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C79">
+        <v>3</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C80">
+        <v>3</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C81">
+        <v>3</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C83">
+        <v>3</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C84">
+        <v>3</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C85">
+        <v>3</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C86">
+        <v>3</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C87">
+        <v>3</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C88">
+        <v>3</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C89">
+        <v>3</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C90">
+        <v>3</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C92">
+        <v>3</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C93">
+        <v>3</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
+      <c r="F93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C94">
+        <v>3</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C95">
+        <v>3</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C96">
+        <v>3</v>
+      </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+      <c r="F96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C97">
+        <v>3</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C98">
+        <v>3</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C99">
+        <v>3</v>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C100">
+        <v>4</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>100</v>
+      </c>
+      <c r="B101" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C101">
+        <v>4</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>101</v>
+      </c>
+      <c r="B102" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C102">
+        <v>5</v>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>102</v>
+      </c>
+      <c r="B103" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C103">
+        <v>5</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+      <c r="F103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>103</v>
+      </c>
+      <c r="B104" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C104">
+        <v>5</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+      <c r="F104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>104</v>
+      </c>
+      <c r="B105" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C105">
+        <v>5</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>105</v>
+      </c>
+      <c r="B106" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C106">
+        <v>5</v>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>106</v>
+      </c>
+      <c r="B107" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C107">
+        <v>5</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>107</v>
+      </c>
+      <c r="B108" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C108">
+        <v>5</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C109">
+        <v>5</v>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C110">
+        <v>5</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C111">
+        <v>5</v>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+      <c r="F111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C112">
+        <v>5</v>
+      </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
+      <c r="F112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C113">
+        <v>5</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113" t="str">
+        <v/>
+      </c>
+      <c r="F113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C114">
+        <v>5</v>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
+      <c r="F114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C115">
+        <v>5</v>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
+      <c r="F115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C116">
+        <v>5</v>
+      </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
+      <c r="F116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C117">
+        <v>5</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
+      <c r="F117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C118">
+        <v>5</v>
+      </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+      <c r="F118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C119">
+        <v>5</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C120">
+        <v>5</v>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+      <c r="F120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C121">
+        <v>5</v>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121" t="str">
+        <v/>
+      </c>
+      <c r="F121" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C122">
+        <v>5</v>
+      </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
+      <c r="E122" t="str">
+        <v/>
+      </c>
+      <c r="F122" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C123">
+        <v>5</v>
+      </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
+      <c r="E123" t="str">
+        <v/>
+      </c>
+      <c r="F123" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C124">
+        <v>5</v>
+      </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
+      <c r="F124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C125">
+        <v>5</v>
+      </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
+      <c r="E125" t="str">
+        <v/>
+      </c>
+      <c r="F125" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C126">
+        <v>5</v>
+      </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
+      <c r="E126" t="str">
+        <v/>
+      </c>
+      <c r="F126" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C127">
+        <v>5</v>
+      </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
+      <c r="E127" t="str">
+        <v/>
+      </c>
+      <c r="F127" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C128">
+        <v>5</v>
+      </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
+      <c r="E128" t="str">
+        <v/>
+      </c>
+      <c r="F128" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C129">
+        <v>5</v>
+      </c>
+      <c r="D129" t="str">
+        <v/>
+      </c>
+      <c r="E129" t="str">
+        <v/>
+      </c>
+      <c r="F129" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C130">
+        <v>5</v>
+      </c>
+      <c r="D130" t="str">
+        <v/>
+      </c>
+      <c r="E130" t="str">
+        <v/>
+      </c>
+      <c r="F130" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C131">
+        <v>5</v>
+      </c>
+      <c r="D131" t="str">
+        <v/>
+      </c>
+      <c r="E131" t="str">
+        <v/>
+      </c>
+      <c r="F131" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C132">
+        <v>5</v>
+      </c>
+      <c r="D132" t="str">
+        <v/>
+      </c>
+      <c r="E132" t="str">
+        <v/>
+      </c>
+      <c r="F132" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C133">
+        <v>5</v>
+      </c>
+      <c r="D133" t="str">
+        <v/>
+      </c>
+      <c r="E133" t="str">
+        <v/>
+      </c>
+      <c r="F133" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C134">
+        <v>5</v>
+      </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
+      <c r="E134" t="str">
+        <v/>
+      </c>
+      <c r="F134" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C135">
+        <v>5</v>
+      </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
+      <c r="E135" t="str">
+        <v/>
+      </c>
+      <c r="F135" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C136">
+        <v>5</v>
+      </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
+      <c r="E136" t="str">
+        <v/>
+      </c>
+      <c r="F136" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C137">
+        <v>4</v>
+      </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
+      <c r="E137" t="str">
+        <v/>
+      </c>
+      <c r="F137" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C138">
+        <v>6</v>
+      </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
+      <c r="E138" t="str">
+        <v/>
+      </c>
+      <c r="F138" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C139">
+        <v>6</v>
+      </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
+      <c r="E139" t="str">
+        <v/>
+      </c>
+      <c r="F139" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C140">
+        <v>6</v>
+      </c>
+      <c r="D140" t="str">
+        <v/>
+      </c>
+      <c r="E140" t="str">
+        <v/>
+      </c>
+      <c r="F140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C141">
+        <v>6</v>
+      </c>
+      <c r="D141" t="str">
+        <v/>
+      </c>
+      <c r="E141" t="str">
+        <v/>
+      </c>
+      <c r="F141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C142">
+        <v>7</v>
+      </c>
+      <c r="D142" t="str">
+        <v/>
+      </c>
+      <c r="E142" t="str">
+        <v/>
+      </c>
+      <c r="F142" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C143">
+        <v>7</v>
+      </c>
+      <c r="D143" t="str">
+        <v/>
+      </c>
+      <c r="E143" t="str">
+        <v/>
+      </c>
+      <c r="F143" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C144">
+        <v>7</v>
+      </c>
+      <c r="D144" t="str">
+        <v/>
+      </c>
+      <c r="E144" t="str">
+        <v/>
+      </c>
+      <c r="F144" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C145">
+        <v>7</v>
+      </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
+      <c r="E145" t="str">
+        <v/>
+      </c>
+      <c r="F145" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C146">
+        <v>7</v>
+      </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
+      <c r="E146" t="str">
+        <v/>
+      </c>
+      <c r="F146" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C147">
+        <v>7</v>
+      </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
+      <c r="E147" t="str">
+        <v/>
+      </c>
+      <c r="F147" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C148">
+        <v>7</v>
+      </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
+      <c r="E148" t="str">
+        <v/>
+      </c>
+      <c r="F148" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C149">
+        <v>7</v>
+      </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
+      <c r="E149" t="str">
+        <v/>
+      </c>
+      <c r="F149" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C150">
+        <v>7</v>
+      </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
+      <c r="E150" t="str">
+        <v/>
+      </c>
+      <c r="F150" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C151">
+        <v>7</v>
+      </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
+      <c r="E151" t="str">
+        <v/>
+      </c>
+      <c r="F151" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C152">
+        <v>7</v>
+      </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
+      <c r="E152" t="str">
+        <v/>
+      </c>
+      <c r="F152" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C153">
+        <v>7</v>
+      </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
+      <c r="E153" t="str">
+        <v/>
+      </c>
+      <c r="F153" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C154">
+        <v>8</v>
+      </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
+      <c r="E154" t="str">
+        <v/>
+      </c>
+      <c r="F154" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C155">
+        <v>8</v>
+      </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
+      <c r="E155" t="str">
+        <v/>
+      </c>
+      <c r="F155" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C156">
+        <v>8</v>
+      </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
+      <c r="E156" t="str">
+        <v/>
+      </c>
+      <c r="F156" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C157">
+        <v>8</v>
+      </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
+      <c r="E157" t="str">
+        <v/>
+      </c>
+      <c r="F157" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C158">
+        <v>8</v>
+      </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
+      <c r="E158" t="str">
+        <v/>
+      </c>
+      <c r="F158" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C159">
+        <v>8</v>
+      </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
+      <c r="E159" t="str">
+        <v/>
+      </c>
+      <c r="F159" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C160">
+        <v>8</v>
+      </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
+      <c r="E160" t="str">
+        <v/>
+      </c>
+      <c r="F160" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C161">
+        <v>8</v>
+      </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
+      <c r="E161" t="str">
+        <v/>
+      </c>
+      <c r="F161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C162">
+        <v>8</v>
+      </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
+      <c r="E162" t="str">
+        <v/>
+      </c>
+      <c r="F162" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C163">
+        <v>8</v>
+      </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
+      <c r="E163" t="str">
+        <v/>
+      </c>
+      <c r="F163" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C164">
+        <v>8</v>
+      </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
+      <c r="E164" t="str">
+        <v/>
+      </c>
+      <c r="F164" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C165">
+        <v>8</v>
+      </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
+      <c r="E165" t="str">
+        <v/>
+      </c>
+      <c r="F165" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C166">
+        <v>8</v>
+      </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
+      <c r="E166" t="str">
+        <v/>
+      </c>
+      <c r="F166" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C167">
+        <v>8</v>
+      </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
+      <c r="E167" t="str">
+        <v/>
+      </c>
+      <c r="F167" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C168">
+        <v>8</v>
+      </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
+      <c r="E168" t="str">
+        <v/>
+      </c>
+      <c r="F168" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C169">
+        <v>8</v>
+      </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
+      <c r="E169" t="str">
+        <v/>
+      </c>
+      <c r="F169" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C170">
+        <v>8</v>
+      </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
+      <c r="E170" t="str">
+        <v/>
+      </c>
+      <c r="F170" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C171">
+        <v>8</v>
+      </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
+      <c r="E171" t="str">
+        <v/>
+      </c>
+      <c r="F171" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C172">
+        <v>9</v>
+      </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
+      <c r="E172" t="str">
+        <v/>
+      </c>
+      <c r="F172" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C173">
+        <v>9</v>
+      </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
+      <c r="E173" t="str">
+        <v/>
+      </c>
+      <c r="F173" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C174">
+        <v>9</v>
+      </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
+      <c r="E174" t="str">
+        <v/>
+      </c>
+      <c r="F174" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C175">
+        <v>9</v>
+      </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
+      <c r="E175" t="str">
+        <v/>
+      </c>
+      <c r="F175" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C176">
+        <v>9</v>
+      </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
+      <c r="E176" t="str">
+        <v/>
+      </c>
+      <c r="F176" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C177">
+        <v>9</v>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+      <c r="E177" t="str">
+        <v/>
+      </c>
+      <c r="F177" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C178">
+        <v>9</v>
+      </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
+      <c r="E178" t="str">
+        <v/>
+      </c>
+      <c r="F178" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C179">
+        <v>9</v>
+      </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
+      <c r="E179" t="str">
+        <v/>
+      </c>
+      <c r="F179" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C180">
+        <v>9</v>
+      </c>
+      <c r="D180" t="str">
+        <v/>
+      </c>
+      <c r="E180" t="str">
+        <v/>
+      </c>
+      <c r="F180" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C181">
+        <v>9</v>
+      </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
+      <c r="E181" t="str">
+        <v/>
+      </c>
+      <c r="F181" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C182">
+        <v>10</v>
+      </c>
+      <c r="D182" t="str">
+        <v/>
+      </c>
+      <c r="E182" t="str">
+        <v/>
+      </c>
+      <c r="F182" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C183">
+        <v>11</v>
+      </c>
+      <c r="D183" t="str">
+        <v/>
+      </c>
+      <c r="E183" t="str">
+        <v/>
+      </c>
+      <c r="F183" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C184">
+        <v>13</v>
+      </c>
+      <c r="D184" t="str">
+        <v/>
+      </c>
+      <c r="E184" t="str">
+        <v/>
+      </c>
+      <c r="F184" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C185">
+        <v>14</v>
+      </c>
+      <c r="D185" t="str">
+        <v/>
+      </c>
+      <c r="E185" t="str">
+        <v/>
+      </c>
+      <c r="F185" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C186">
+        <v>18</v>
+      </c>
+      <c r="D186" t="str">
+        <v/>
+      </c>
+      <c r="E186" t="str">
+        <v/>
+      </c>
+      <c r="F186" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C187">
+        <v>17</v>
+      </c>
+      <c r="D187" t="str">
+        <v/>
+      </c>
+      <c r="E187" t="str">
+        <v/>
+      </c>
+      <c r="F187" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C188">
+        <v>18</v>
+      </c>
+      <c r="D188" t="str">
+        <v/>
+      </c>
+      <c r="E188" t="str">
+        <v/>
+      </c>
+      <c r="F188" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C189">
+        <v>20</v>
+      </c>
+      <c r="D189" t="str">
+        <v/>
+      </c>
+      <c r="E189" t="str">
+        <v/>
+      </c>
+      <c r="F189" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C190">
+        <v>22</v>
+      </c>
+      <c r="D190" t="str">
+        <v/>
+      </c>
+      <c r="E190" t="str">
+        <v/>
+      </c>
+      <c r="F190" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C191">
+        <v>24</v>
+      </c>
+      <c r="D191" t="str">
+        <v/>
+      </c>
+      <c r="E191" t="str">
+        <v/>
+      </c>
+      <c r="F191" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C192">
+        <v>27</v>
+      </c>
+      <c r="D192" t="str">
+        <v/>
+      </c>
+      <c r="E192" t="str">
+        <v/>
+      </c>
+      <c r="F192" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C193">
+        <v>29</v>
+      </c>
+      <c r="D193" t="str">
+        <v/>
+      </c>
+      <c r="E193" t="str">
+        <v/>
+      </c>
+      <c r="F193" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C194">
+        <v>32</v>
+      </c>
+      <c r="D194" t="str">
+        <v/>
+      </c>
+      <c r="E194" t="str">
+        <v/>
+      </c>
+      <c r="F194" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C195">
+        <v>35</v>
+      </c>
+      <c r="D195" t="str">
+        <v/>
+      </c>
+      <c r="E195" t="str">
+        <v/>
+      </c>
+      <c r="F195" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C196">
+        <v>39</v>
+      </c>
+      <c r="D196" t="str">
+        <v/>
+      </c>
+      <c r="E196" t="str">
+        <v/>
+      </c>
+      <c r="F196" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C197">
+        <v>43</v>
+      </c>
+      <c r="D197" t="str">
+        <v/>
+      </c>
+      <c r="E197" t="str">
+        <v/>
+      </c>
+      <c r="F197" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C198">
+        <v>48</v>
+      </c>
+      <c r="D198" t="str">
+        <v/>
+      </c>
+      <c r="E198" t="str">
+        <v/>
+      </c>
+      <c r="F198" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C199">
+        <v>52</v>
+      </c>
+      <c r="D199" t="str">
+        <v/>
+      </c>
+      <c r="E199" t="str">
+        <v/>
+      </c>
+      <c r="F199" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C200">
+        <v>59</v>
+      </c>
+      <c r="D200" t="str">
+        <v/>
+      </c>
+      <c r="E200" t="str">
+        <v/>
+      </c>
+      <c r="F200" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="str">
+        <v>MK V</v>
+      </c>
+      <c r="C201">
+        <v>64</v>
+      </c>
+      <c r="D201" t="str">
+        <v/>
+      </c>
+      <c r="E201" t="str">
+        <v/>
+      </c>
+      <c r="F201" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F201"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>